<commit_message>
added errormessage for login
</commit_message>
<xml_diff>
--- a/WebAutomationAssignment/Data Files/LoginPayloads.xlsx
+++ b/WebAutomationAssignment/Data Files/LoginPayloads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/willyhsu0130/Documents/Humber/Semester4/WebApp/GrapherProj/WebAutomationAssignment/Data Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{58052E96-B796-D342-B71C-537AE2BFF7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD89D244-AD03-294E-B30E-3CFD7B1AB46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" xr2:uid="{59698CEE-0845-2744-B554-640FF60A9BC6}"/>
   </bookViews>
@@ -38,12 +38,67 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>willyhsu0130</t>
+  </si>
+  <si>
+    <t>willyhsu0130@gmail.com</t>
+  </si>
+  <si>
+    <t>WILLYHSU0130</t>
+  </si>
+  <si>
+    <t>willyhsu013</t>
+  </si>
+  <si>
+    <t>isSuccess</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Password Empty</t>
+  </si>
+  <si>
+    <t>Username empty</t>
+  </si>
+  <si>
+    <t>account is not registered</t>
+  </si>
+  <si>
+    <t>registered username but in upper case</t>
+  </si>
+  <si>
+    <t>registered email</t>
+  </si>
+  <si>
+    <t>registered username</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -66,13 +121,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -405,9 +463,110 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31C06AFE-44CC-B14C-AEA4-770FEC0486E4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="30.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>12345678</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>12345678</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>12345678</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>12345678</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>12345678</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{E29C7003-9C15-8A41-99BB-06FF88F2A3E1}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>